<commit_message>
Penyesuaian layout Create PR dengan template baru, penambahan tampilan TvDashboard, penambahan bar gauge pada laporan analitik
</commit_message>
<xml_diff>
--- a/Templates/Format_PR.xlsx
+++ b/Templates/Format_PR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DashboardTeknikP1\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B972FF76-FC68-41F1-921B-1F33306C9876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201EC1A5-9FAA-49D8-BD60-B9EB82C8DA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{DDF71227-D3ED-492C-8E4C-2B72C9515BF4}"/>
   </bookViews>
@@ -34,35 +34,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>Quantity</t>
-  </si>
-  <si>
     <t>Satuan</t>
   </si>
   <si>
-    <t>Deskripsi Barang</t>
-  </si>
-  <si>
-    <t>No Material</t>
-  </si>
-  <si>
-    <t>Delivery</t>
-  </si>
-  <si>
-    <t>G/L Acc</t>
-  </si>
-  <si>
-    <t>Cost Center / WBS Element</t>
-  </si>
-  <si>
-    <t>Remark</t>
-  </si>
-  <si>
     <t>PLEASE ORDER THE FOLLOWING MATERIAL</t>
   </si>
   <si>
@@ -81,49 +60,73 @@
     <t>No. Terbitan</t>
   </si>
   <si>
-    <t>: PURCH - 002</t>
-  </si>
-  <si>
-    <t>: 1.0</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
     <t>Delivery To</t>
   </si>
   <si>
     <t>: (1108) PT. ISM Tbk, Cibitung</t>
   </si>
   <si>
-    <t>Purchasing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Received By : </t>
-  </si>
-  <si>
     <t>Requisitioner :</t>
   </si>
   <si>
-    <t>Dept User</t>
-  </si>
-  <si>
     <t>Reviewed :</t>
   </si>
   <si>
     <t>(…..............................)</t>
   </si>
   <si>
-    <t>Accounting</t>
-  </si>
-  <si>
     <t xml:space="preserve">Approved by : </t>
   </si>
   <si>
-    <t>Dept. Head</t>
+    <t>Material</t>
+  </si>
+  <si>
+    <t>Description of Goods</t>
+  </si>
+  <si>
+    <t>QTY</t>
+  </si>
+  <si>
+    <t>Delivery Date</t>
+  </si>
+  <si>
+    <t>Stok di SAP Update      (Cek MD04)</t>
+  </si>
+  <si>
+    <t>Apa ada PR/PO outstanding?           (Cek MD04)</t>
+  </si>
+  <si>
+    <t>Storage Location</t>
+  </si>
+  <si>
+    <t>Kebutuhan Minimal Stok</t>
+  </si>
+  <si>
+    <t>Keterangan</t>
+  </si>
+  <si>
+    <t>: Tech - 002</t>
+  </si>
+  <si>
+    <t>: 4.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checked By : </t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Sect. Tek</t>
+  </si>
+  <si>
+    <t>FTM</t>
+  </si>
+  <si>
+    <t>SUMANTRI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPV Tek </t>
   </si>
 </sst>
 </file>
@@ -163,7 +166,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -470,28 +473,82 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -512,15 +569,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
@@ -533,34 +581,75 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -881,568 +970,527 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.77734375" customWidth="1"/>
-    <col min="2" max="4" width="4.21875" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" customWidth="1"/>
-    <col min="6" max="6" width="34.44140625" customWidth="1"/>
-    <col min="9" max="9" width="17.77734375" customWidth="1"/>
-    <col min="11" max="11" width="11.77734375" customWidth="1"/>
+    <col min="2" max="2" width="4.21875" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" customWidth="1"/>
+    <col min="4" max="4" width="34.44140625" customWidth="1"/>
+    <col min="7" max="7" width="17.77734375" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="11" width="10.6640625" customWidth="1"/>
     <col min="12" max="12" width="42.77734375" customWidth="1"/>
     <col min="13" max="13" width="3.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="4"/>
-      <c r="L2" s="5" t="s">
+      <c r="B2" s="40" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="3"/>
+    </row>
+    <row r="3" spans="2:12" ht="19.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="33" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" spans="2:12" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="39" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="39"/>
+    </row>
+    <row r="5" spans="2:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="35" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="38"/>
+    </row>
+    <row r="6" spans="2:12" s="1" customFormat="1" ht="47.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="2:12" ht="19.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" s="7"/>
-      <c r="L3" s="8" t="s">
+      <c r="E6" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="2:12" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" spans="2:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="16"/>
-    </row>
-    <row r="6" spans="2:12" s="1" customFormat="1" ht="47.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="11" t="s">
+      <c r="F6" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="H6" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="I6" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="K6" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="L6" s="13" t="s">
-        <v>8</v>
+      <c r="I6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="19"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="13"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B8" s="20"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="21"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="31"/>
+      <c r="L8" s="15"/>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="20"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="21"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="15"/>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B10" s="20"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="21"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="15"/>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B11" s="20"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="21"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="15"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B12" s="20"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="21"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="15"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B13" s="20"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="21"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="15"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B14" s="20"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="21"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="15"/>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B15" s="20"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="21"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="15"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B16" s="20"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="21"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="15"/>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B17" s="20"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="21"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="15"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B18" s="20"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="21"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="15"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B19" s="20"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="21"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="15"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B20" s="20"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="21"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="15"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B21" s="20"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-      <c r="L21" s="21"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="15"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B22" s="20"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="21"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="15"/>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B23" s="20"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="21"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
+      <c r="L23" s="15"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B24" s="20"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="21"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="15"/>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B25" s="20"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
-      <c r="L25" s="21"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="31"/>
+      <c r="K25" s="31"/>
+      <c r="L25" s="15"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B26" s="20"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="9"/>
-      <c r="L26" s="21"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="15"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B27" s="20"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
-      <c r="L27" s="21"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="31"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="15"/>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B28" s="20"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="21"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="15"/>
     </row>
     <row r="29" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="22"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23"/>
-      <c r="K29" s="23"/>
-      <c r="L29" s="24"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="32"/>
+      <c r="L29" s="18"/>
     </row>
     <row r="30" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="31" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B31" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="28"/>
+      <c r="B31" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="20"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="21"/>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B32" s="29"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="31"/>
+      <c r="B32" s="22"/>
+      <c r="L32" s="23"/>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B33" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="H33" s="33"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="33" t="s">
+      <c r="B33" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="K33" s="33"/>
-      <c r="L33" s="34" t="s">
+      <c r="C33" s="44"/>
+      <c r="E33" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" s="44"/>
+      <c r="H33" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="I33" s="44"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="24"/>
+      <c r="L33" s="25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B34" s="22"/>
+      <c r="L34" s="23"/>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B35" s="22"/>
+      <c r="L35" s="23"/>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B36" s="22"/>
+      <c r="L36" s="23"/>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B37" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="44"/>
+      <c r="E37" s="48"/>
+      <c r="F37" s="48"/>
+      <c r="H37" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I37" s="44"/>
+      <c r="J37" s="24"/>
+      <c r="K37" s="24"/>
+      <c r="L37" s="25" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="C38" s="45"/>
+      <c r="D38" s="27"/>
+      <c r="E38" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F38" s="45"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="45" t="s">
+        <v>30</v>
+      </c>
+      <c r="I38" s="45"/>
+      <c r="J38" s="26"/>
+      <c r="K38" s="26"/>
+      <c r="L38" s="28" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B34" s="29"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
-      <c r="I34" s="30"/>
-      <c r="J34" s="30"/>
-      <c r="K34" s="30"/>
-      <c r="L34" s="31"/>
-    </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B35" s="29"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="30"/>
-      <c r="E35" s="30"/>
-      <c r="F35" s="30"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="30"/>
-      <c r="I35" s="30"/>
-      <c r="J35" s="30"/>
-      <c r="K35" s="30"/>
-      <c r="L35" s="31"/>
-    </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B36" s="29"/>
-      <c r="C36" s="30"/>
-      <c r="D36" s="30"/>
-      <c r="E36" s="30"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="30"/>
-      <c r="J36" s="30"/>
-      <c r="K36" s="30"/>
-      <c r="L36" s="31"/>
-    </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B37" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="35"/>
-      <c r="H37" s="35"/>
-      <c r="I37" s="30"/>
-      <c r="J37" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="K37" s="33"/>
-      <c r="L37" s="34" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="38" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="37"/>
-      <c r="F38" s="38"/>
-      <c r="G38" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="H38" s="37"/>
-      <c r="I38" s="38"/>
-      <c r="J38" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="K38" s="37"/>
-      <c r="L38" s="39" t="s">
-        <v>29</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="J5:L5"/>
+  <mergeCells count="14">
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="H5:L5"/>
     <mergeCell ref="B4:L4"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="75" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix bug logout tv dashboard, penambahan slide daftar temuan di tv dashboard, fix bug darkmode 2
</commit_message>
<xml_diff>
--- a/Templates/Format_PR.xlsx
+++ b/Templates/Format_PR.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DashboardTeknikP1\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DashboardTeknikP1_Data_Xlsx\Publish_Server\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201EC1A5-9FAA-49D8-BD60-B9EB82C8DA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B4150F-09C6-4386-87FB-2FF470365017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{DDF71227-D3ED-492C-8E4C-2B72C9515BF4}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>No</t>
   </si>
@@ -60,12 +60,6 @@
     <t>No. Terbitan</t>
   </si>
   <si>
-    <t>Delivery To</t>
-  </si>
-  <si>
-    <t>: (1108) PT. ISM Tbk, Cibitung</t>
-  </si>
-  <si>
     <t>Requisitioner :</t>
   </si>
   <si>
@@ -93,9 +87,6 @@
     <t>Stok di SAP Update      (Cek MD04)</t>
   </si>
   <si>
-    <t>Apa ada PR/PO outstanding?           (Cek MD04)</t>
-  </si>
-  <si>
     <t>Storage Location</t>
   </si>
   <si>
@@ -127,6 +118,13 @@
   </si>
   <si>
     <t xml:space="preserve">SPV Tek </t>
+  </si>
+  <si>
+    <t>Delivery To : (1108) PT. ISM Tbk, Cibitung</t>
+  </si>
+  <si>
+    <t>Apa ada PR/PO outstanding?
+(Cek MD04)</t>
   </si>
 </sst>
 </file>
@@ -540,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -578,9 +576,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
@@ -610,6 +605,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -637,20 +647,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -983,106 +984,106 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="34" t="s">
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="34" t="s">
-        <v>23</v>
+      <c r="I2" s="33" t="s">
+        <v>20</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="3"/>
     </row>
     <row r="3" spans="2:12" ht="19.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="33" t="s">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="33" t="s">
-        <v>24</v>
+      <c r="I3" s="32" t="s">
+        <v>21</v>
       </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="5"/>
     </row>
     <row r="4" spans="2:12" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="43"/>
+      <c r="J4" s="43"/>
+      <c r="K4" s="43"/>
+      <c r="L4" s="43"/>
     </row>
     <row r="5" spans="2:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
-      <c r="L5" s="38"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="42"/>
     </row>
     <row r="6" spans="2:12" s="1" customFormat="1" ht="47.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="7" t="s">
         <v>0</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>14</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>16</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>1</v>
       </c>
       <c r="G6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="J6" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="K6" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="L6" s="10" t="s">
         <v>19</v>
-      </c>
-      <c r="J6" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="K6" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="L6" s="10" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
@@ -1094,8 +1095,8 @@
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="30"/>
+      <c r="J7" s="29"/>
+      <c r="K7" s="29"/>
       <c r="L7" s="13"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
@@ -1107,8 +1108,8 @@
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="31"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
       <c r="L8" s="15"/>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
@@ -1120,8 +1121,8 @@
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
       <c r="L9" s="15"/>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
@@ -1133,8 +1134,8 @@
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="31"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
       <c r="L10" s="15"/>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.3">
@@ -1146,8 +1147,8 @@
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="31"/>
+      <c r="J11" s="30"/>
+      <c r="K11" s="30"/>
       <c r="L11" s="15"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
@@ -1159,8 +1160,8 @@
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
-      <c r="J12" s="31"/>
-      <c r="K12" s="31"/>
+      <c r="J12" s="30"/>
+      <c r="K12" s="30"/>
       <c r="L12" s="15"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.3">
@@ -1172,8 +1173,8 @@
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="31"/>
+      <c r="J13" s="30"/>
+      <c r="K13" s="30"/>
       <c r="L13" s="15"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
@@ -1185,8 +1186,8 @@
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
+      <c r="J14" s="30"/>
+      <c r="K14" s="30"/>
       <c r="L14" s="15"/>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.3">
@@ -1198,8 +1199,8 @@
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
-      <c r="J15" s="31"/>
-      <c r="K15" s="31"/>
+      <c r="J15" s="30"/>
+      <c r="K15" s="30"/>
       <c r="L15" s="15"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.3">
@@ -1211,8 +1212,8 @@
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="31"/>
-      <c r="K16" s="31"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
       <c r="L16" s="15"/>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.3">
@@ -1224,8 +1225,8 @@
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="31"/>
+      <c r="J17" s="30"/>
+      <c r="K17" s="30"/>
       <c r="L17" s="15"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.3">
@@ -1237,8 +1238,8 @@
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
       <c r="L18" s="15"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.3">
@@ -1250,8 +1251,8 @@
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="31"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="30"/>
       <c r="L19" s="15"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.3">
@@ -1263,8 +1264,8 @@
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
       <c r="L20" s="15"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.3">
@@ -1276,8 +1277,8 @@
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
-      <c r="J21" s="31"/>
-      <c r="K21" s="31"/>
+      <c r="J21" s="30"/>
+      <c r="K21" s="30"/>
       <c r="L21" s="15"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.3">
@@ -1289,8 +1290,8 @@
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
-      <c r="J22" s="31"/>
-      <c r="K22" s="31"/>
+      <c r="J22" s="30"/>
+      <c r="K22" s="30"/>
       <c r="L22" s="15"/>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.3">
@@ -1302,8 +1303,8 @@
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
       <c r="I23" s="6"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31"/>
+      <c r="J23" s="30"/>
+      <c r="K23" s="30"/>
       <c r="L23" s="15"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.3">
@@ -1315,8 +1316,8 @@
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
-      <c r="J24" s="31"/>
-      <c r="K24" s="31"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="30"/>
       <c r="L24" s="15"/>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.3">
@@ -1328,8 +1329,8 @@
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
       <c r="I25" s="6"/>
-      <c r="J25" s="31"/>
-      <c r="K25" s="31"/>
+      <c r="J25" s="30"/>
+      <c r="K25" s="30"/>
       <c r="L25" s="15"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.3">
@@ -1341,8 +1342,8 @@
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
       <c r="I26" s="6"/>
-      <c r="J26" s="31"/>
-      <c r="K26" s="31"/>
+      <c r="J26" s="30"/>
+      <c r="K26" s="30"/>
       <c r="L26" s="15"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.3">
@@ -1354,8 +1355,8 @@
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
       <c r="I27" s="6"/>
-      <c r="J27" s="31"/>
-      <c r="K27" s="31"/>
+      <c r="J27" s="30"/>
+      <c r="K27" s="30"/>
       <c r="L27" s="15"/>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.3">
@@ -1367,8 +1368,8 @@
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
       <c r="I28" s="6"/>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
       <c r="L28" s="15"/>
     </row>
     <row r="29" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1380,103 +1381,107 @@
       <c r="G29" s="17"/>
       <c r="H29" s="17"/>
       <c r="I29" s="17"/>
-      <c r="J29" s="32"/>
-      <c r="K29" s="32"/>
+      <c r="J29" s="31"/>
+      <c r="K29" s="31"/>
       <c r="L29" s="18"/>
     </row>
     <row r="30" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="31" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" s="49"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="19"/>
+      <c r="L31" s="20"/>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B32" s="21"/>
+      <c r="L32" s="22"/>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B33" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C33" s="34"/>
+      <c r="E33" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C31" s="20" t="s">
+      <c r="F33" s="34"/>
+      <c r="H33" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
-      <c r="L31" s="21"/>
-    </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B32" s="22"/>
-      <c r="L32" s="23"/>
-    </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B33" s="46" t="s">
+      <c r="I33" s="34"/>
+      <c r="J33" s="23"/>
+      <c r="K33" s="23"/>
+      <c r="L33" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B34" s="21"/>
+      <c r="L34" s="22"/>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B35" s="21"/>
+      <c r="L35" s="22"/>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B36" s="21"/>
+      <c r="L36" s="22"/>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B37" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="34"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="H37" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="I37" s="34"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="C38" s="35"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="F38" s="35"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="I38" s="35"/>
+      <c r="J38" s="25"/>
+      <c r="K38" s="25"/>
+      <c r="L38" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="44"/>
-      <c r="E33" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="F33" s="44"/>
-      <c r="H33" s="44" t="s">
-        <v>11</v>
-      </c>
-      <c r="I33" s="44"/>
-      <c r="J33" s="24"/>
-      <c r="K33" s="24"/>
-      <c r="L33" s="25" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B34" s="22"/>
-      <c r="L34" s="23"/>
-    </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B35" s="22"/>
-      <c r="L35" s="23"/>
-    </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B36" s="22"/>
-      <c r="L36" s="23"/>
-    </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B37" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" s="44"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
-      <c r="H37" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="I37" s="44"/>
-      <c r="J37" s="24"/>
-      <c r="K37" s="24"/>
-      <c r="L37" s="25" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="38" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="47" t="s">
-        <v>26</v>
-      </c>
-      <c r="C38" s="45"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F38" s="45"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="45" t="s">
-        <v>30</v>
-      </c>
-      <c r="I38" s="45"/>
-      <c r="J38" s="26"/>
-      <c r="K38" s="26"/>
-      <c r="L38" s="28" t="s">
-        <v>28</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="H5:L5"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B3:G3"/>
     <mergeCell ref="H33:I33"/>
     <mergeCell ref="H37:I37"/>
     <mergeCell ref="H38:I38"/>
@@ -1486,11 +1491,6 @@
     <mergeCell ref="E33:F33"/>
     <mergeCell ref="E37:F37"/>
     <mergeCell ref="E38:F38"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="H5:L5"/>
-    <mergeCell ref="B4:L4"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="75" orientation="landscape" r:id="rId1"/>

</xml_diff>